<commit_message>
April 2026 - Update
</commit_message>
<xml_diff>
--- a/April 2026.xlsx
+++ b/April 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abutalib/Projects/personal-accounting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E3F0BF-A198-C740-872A-26EBCF74928B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C2814E-17BB-DC4E-A759-B1EFDB9BDEEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
   </bookViews>
   <sheets>
     <sheet name="مصاريف الشهر" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="157">
   <si>
     <t>فاتورة الكهرباء</t>
   </si>
@@ -505,6 +505,9 @@
   </si>
   <si>
     <t>تذكرة عودة مصر</t>
+  </si>
+  <si>
+    <t>إيجار شقة 19 يوم</t>
   </si>
 </sst>
 </file>
@@ -647,13 +650,13 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1056,14 +1059,14 @@
       <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19" t="s">
+      <c r="F1" s="20"/>
+      <c r="G1" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="19"/>
+      <c r="H1" s="20"/>
       <c r="I1" s="4"/>
       <c r="J1" s="3" t="s">
         <v>17</v>
@@ -1124,7 +1127,7 @@
       </c>
       <c r="W2" s="3">
         <f>SUM(W7:W16)</f>
-        <v>9932</v>
+        <v>7698</v>
       </c>
       <c r="X2" s="4"/>
       <c r="Y2" s="3" t="s">
@@ -1132,7 +1135,7 @@
       </c>
       <c r="AA2" s="3">
         <f>SUM(AA7:AB35)</f>
-        <v>23589</v>
+        <v>21355</v>
       </c>
       <c r="AB2" s="4"/>
       <c r="AC2" s="3" t="s">
@@ -1256,10 +1259,10 @@
       <c r="O6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P6" s="18" t="s">
+      <c r="P6" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="Q6" s="18"/>
+      <c r="Q6" s="19"/>
       <c r="R6" s="9"/>
       <c r="U6" s="9"/>
       <c r="X6" s="9"/>
@@ -1583,7 +1586,7 @@
       </c>
       <c r="W12" s="3">
         <f>J32</f>
-        <v>6068</v>
+        <v>3834</v>
       </c>
       <c r="X12" s="4"/>
       <c r="AB12" s="4"/>
@@ -2075,7 +2078,7 @@
       </c>
       <c r="AA31" s="3">
         <f>W2</f>
-        <v>9932</v>
+        <v>7698</v>
       </c>
       <c r="AB31" s="3"/>
     </row>
@@ -2091,7 +2094,7 @@
       <c r="I32" s="3"/>
       <c r="J32" s="3">
         <f>الأرصدة!M29-'مصاريف الشهر'!D32</f>
-        <v>6068</v>
+        <v>3834</v>
       </c>
       <c r="O32" s="3">
         <f>E3</f>
@@ -2103,7 +2106,7 @@
       </c>
       <c r="Q32" s="3">
         <f>J32-SUM(O32:P32)</f>
-        <v>-1584</v>
+        <v>-3818</v>
       </c>
       <c r="R32" s="3"/>
       <c r="U32" s="3"/>
@@ -2251,7 +2254,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F05345A-5E98-0C43-BBDD-1D2CC38375ED}">
-  <dimension ref="A1:AJ31"/>
+  <dimension ref="A1:AG31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -2277,8 +2280,8 @@
     <col min="21" max="21" width="10.1640625" customWidth="1"/>
     <col min="22" max="22" width="0.1640625" customWidth="1"/>
     <col min="23" max="23" width="10.83203125" customWidth="1"/>
-    <col min="24" max="24" width="29.33203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="28.83203125" customWidth="1"/>
+    <col min="25" max="25" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="0.5" customWidth="1"/>
     <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="20" bestFit="1" customWidth="1"/>
@@ -2368,7 +2371,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="11">
         <f>SUM(J6:J11)</f>
-        <v>6300</v>
+        <v>5800</v>
       </c>
       <c r="K2" s="4"/>
       <c r="L2" s="11">
@@ -2384,13 +2387,13 @@
       <c r="R2" s="4"/>
       <c r="S2" s="11">
         <f>SUM(U6:U19)</f>
-        <v>33671</v>
+        <v>36405</v>
       </c>
       <c r="T2" s="11"/>
       <c r="V2" s="2"/>
       <c r="W2" s="11">
         <f>SUM(Y6:Y20)</f>
-        <v>6448</v>
+        <v>9182</v>
       </c>
       <c r="X2" s="11">
         <f>1500+(303*3)</f>
@@ -2398,7 +2401,7 @@
       </c>
       <c r="Y2" s="11">
         <f>SUM(W2:X2)</f>
-        <v>8857</v>
+        <v>11591</v>
       </c>
       <c r="Z2" s="4"/>
       <c r="AA2" s="11">
@@ -2804,7 +2807,7 @@
         <v>32</v>
       </c>
       <c r="J9" s="11">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="3">
@@ -3312,18 +3315,24 @@
       <c r="S18" s="3">
         <v>4</v>
       </c>
-      <c r="T18" s="20" t="str">
+      <c r="T18" s="18" t="str">
         <f>W1</f>
         <v>سفرة مصر</v>
       </c>
       <c r="U18" s="11">
         <f>W2</f>
-        <v>6448</v>
+        <v>9182</v>
       </c>
       <c r="V18" s="2"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
-      <c r="Y18" s="11"/>
+      <c r="W18" s="3">
+        <v>10</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="Y18" s="11">
+        <v>2734</v>
+      </c>
       <c r="Z18" s="4"/>
       <c r="AA18" s="3"/>
       <c r="AB18" s="3"/>
@@ -3473,7 +3482,7 @@
       </c>
       <c r="M23" s="6">
         <f>O2-S2</f>
-        <v>29381</v>
+        <v>26647</v>
       </c>
       <c r="N23" s="4"/>
       <c r="O23" s="3"/>
@@ -3551,7 +3560,7 @@
       </c>
       <c r="M26" s="6">
         <f>-I2</f>
-        <v>-6300</v>
+        <v>-5800</v>
       </c>
       <c r="N26" s="4"/>
       <c r="O26" s="3"/>
@@ -3594,7 +3603,7 @@
       </c>
       <c r="Y27" s="12">
         <f>M29-W27</f>
-        <v>-8977</v>
+        <v>-11211</v>
       </c>
     </row>
     <row r="28" spans="2:33" ht="22" x14ac:dyDescent="0.3">
@@ -3638,7 +3647,7 @@
       </c>
       <c r="M29" s="6">
         <f>SUM(M23:M28)</f>
-        <v>26289</v>
+        <v>24055</v>
       </c>
       <c r="N29" s="4"/>
       <c r="O29" s="3"/>

</xml_diff>

<commit_message>
April 2026 - Finalized
</commit_message>
<xml_diff>
--- a/April 2026.xlsx
+++ b/April 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abutalib/Projects/personal-accounting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C2814E-17BB-DC4E-A759-B1EFDB9BDEEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A398737A-5BAB-C641-8DEB-C8865F9944DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
   </bookViews>
   <sheets>
     <sheet name="مصاريف الشهر" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="149">
   <si>
     <t>فاتورة الكهرباء</t>
   </si>
@@ -171,9 +171,6 @@
     <t>رسوم التسجيل للجامعة</t>
   </si>
   <si>
-    <t>مصروف</t>
-  </si>
-  <si>
     <t>تحويلات حساب الادخار</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>ادخار إضافي</t>
   </si>
   <si>
-    <t>الماك</t>
-  </si>
-  <si>
     <t>تفاصيل</t>
   </si>
   <si>
@@ -348,18 +342,12 @@
     <t>صدقة مؤيد</t>
   </si>
   <si>
-    <t>ثياب</t>
-  </si>
-  <si>
     <t>عملية القسطرة لأبوي</t>
   </si>
   <si>
     <t>تصليح السيارة</t>
   </si>
   <si>
-    <t>علاج إرشاد</t>
-  </si>
-  <si>
     <t>الراجحي</t>
   </si>
   <si>
@@ -381,42 +369,6 @@
     <t>تصليح الكامري</t>
   </si>
   <si>
-    <t>تصليح الماك</t>
-  </si>
-  <si>
-    <t>حلاقة ومصاريف عيد</t>
-  </si>
-  <si>
-    <t>صدقات</t>
-  </si>
-  <si>
-    <t>طلعة هشام</t>
-  </si>
-  <si>
-    <t>عطر وسحور</t>
-  </si>
-  <si>
-    <t>عيدية منى</t>
-  </si>
-  <si>
-    <t>غدا العيد</t>
-  </si>
-  <si>
-    <t>قسط كنبة</t>
-  </si>
-  <si>
-    <t>ملابس صيف</t>
-  </si>
-  <si>
-    <t>ألعاب أطفال للعيد</t>
-  </si>
-  <si>
-    <t>شغالة باليوم</t>
-  </si>
-  <si>
-    <t>تجديد جواز منى</t>
-  </si>
-  <si>
     <t>قسط الجامعة 2- الفصل 1</t>
   </si>
   <si>
@@ -480,9 +432,6 @@
     <t>نثريات سفر</t>
   </si>
   <si>
-    <t>العملية 1500 متوقع</t>
-  </si>
-  <si>
     <t>أقساط</t>
   </si>
   <si>
@@ -508,6 +457,33 @@
   </si>
   <si>
     <t>إيجار شقة 19 يوم</t>
+  </si>
+  <si>
+    <t>الجهة</t>
+  </si>
+  <si>
+    <t>تمارا</t>
+  </si>
+  <si>
+    <t>تابي</t>
+  </si>
+  <si>
+    <t>فرق تذكرة العودة</t>
+  </si>
+  <si>
+    <t>مصاريف</t>
+  </si>
+  <si>
+    <t>رسوم الفحص</t>
+  </si>
+  <si>
+    <t>العملية  4,951  متوقع</t>
+  </si>
+  <si>
+    <t>اسكندرية</t>
+  </si>
+  <si>
+    <t>قسط الراجحي</t>
   </si>
 </sst>
 </file>
@@ -585,7 +561,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -627,7 +603,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -645,11 +621,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -657,6 +628,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1013,7 +991,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C2F52D6-F91F-A540-B517-60C5A16A2B32}">
-  <dimension ref="A1:AF45"/>
+  <dimension ref="A1:AF46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="22" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" style="3" bestFit="1" customWidth="1"/>
@@ -1053,39 +1031,39 @@
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="H1" s="20"/>
+      <c r="E1" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="H1" s="17"/>
       <c r="I1" s="4"/>
       <c r="J1" s="3" t="s">
         <v>17</v>
       </c>
       <c r="R1" s="4"/>
       <c r="S1" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="U1" s="4"/>
       <c r="V1" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="X1" s="4"/>
       <c r="Y1" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="AB1" s="4"/>
       <c r="AC1" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -1094,16 +1072,16 @@
       </c>
       <c r="C2" s="4"/>
       <c r="E2" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="3" t="s">
@@ -1111,7 +1089,7 @@
       </c>
       <c r="O2" s="3">
         <f>SUM(O7:O26)</f>
-        <v>4016</v>
+        <v>5917</v>
       </c>
       <c r="R2" s="4"/>
       <c r="S2" s="3" t="s">
@@ -1119,7 +1097,7 @@
       </c>
       <c r="T2" s="3">
         <f>SUM(T7:T16)</f>
-        <v>595</v>
+        <v>0</v>
       </c>
       <c r="U2" s="4"/>
       <c r="V2" s="3" t="s">
@@ -1127,7 +1105,7 @@
       </c>
       <c r="W2" s="3">
         <f>SUM(W7:W16)</f>
-        <v>7698</v>
+        <v>20154</v>
       </c>
       <c r="X2" s="4"/>
       <c r="Y2" s="3" t="s">
@@ -1135,7 +1113,7 @@
       </c>
       <c r="AA2" s="3">
         <f>SUM(AA7:AB35)</f>
-        <v>21355</v>
+        <v>35298</v>
       </c>
       <c r="AB2" s="4"/>
       <c r="AC2" s="3" t="s">
@@ -1157,11 +1135,11 @@
       </c>
       <c r="E3" s="3">
         <f>SUM(E7:E25)</f>
-        <v>2007</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3">
         <f>SUM(F7:F28)</f>
-        <v>5645</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3">
         <f>SUM(G7:G25)</f>
@@ -1169,7 +1147,7 @@
       </c>
       <c r="H3" s="3">
         <f>SUM(H7:H25)</f>
-        <v>2595</v>
+        <v>2000</v>
       </c>
       <c r="I3" s="4"/>
       <c r="R3" s="4"/>
@@ -1182,13 +1160,13 @@
       </c>
       <c r="AD3" s="3">
         <f>AA21-AD2</f>
-        <v>226</v>
+        <v>380</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.3">
       <c r="C4" s="4"/>
       <c r="D4" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E4" s="3">
         <f>B11</f>
@@ -1200,11 +1178,11 @@
       </c>
       <c r="G4" s="3">
         <f>E5</f>
-        <v>-423</v>
+        <v>-317</v>
       </c>
       <c r="H4" s="3">
         <f>F5</f>
-        <v>3382</v>
+        <v>9027</v>
       </c>
       <c r="I4" s="4"/>
       <c r="R4" s="4"/>
@@ -1220,19 +1198,19 @@
       </c>
       <c r="E5" s="3">
         <f>E4-O2-E3</f>
-        <v>-423</v>
+        <v>-317</v>
       </c>
       <c r="F5" s="3">
         <f>F4-F3</f>
-        <v>3382</v>
+        <v>9027</v>
       </c>
       <c r="G5" s="3">
         <f>G4-G3</f>
-        <v>-423</v>
+        <v>-317</v>
       </c>
       <c r="H5" s="3">
         <f>H4-H3</f>
-        <v>787</v>
+        <v>7027</v>
       </c>
       <c r="I5" s="4"/>
       <c r="R5" s="4"/>
@@ -1245,24 +1223,24 @@
       <c r="C6" s="9"/>
       <c r="I6" s="9"/>
       <c r="K6" s="8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P6" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q6" s="19"/>
+      <c r="P6" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q6" s="16"/>
       <c r="R6" s="9"/>
       <c r="U6" s="9"/>
       <c r="X6" s="9"/>
@@ -1270,43 +1248,34 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B7" s="3">
         <v>800</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1600</v>
-      </c>
       <c r="I7" s="4"/>
       <c r="J7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="M7" s="3">
         <f>SUM(N7:O7)</f>
-        <v>134</v>
+        <v>395</v>
       </c>
       <c r="O7" s="3">
         <f>SUM(P7:Q7)</f>
-        <v>134</v>
+        <v>395</v>
+      </c>
+      <c r="P7" s="3">
+        <v>290</v>
       </c>
       <c r="Q7" s="3">
-        <v>134</v>
+        <v>105</v>
       </c>
       <c r="R7" s="4"/>
-      <c r="S7" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="T7" s="3">
-        <v>64</v>
-      </c>
       <c r="U7" s="4"/>
       <c r="V7" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="W7" s="3">
         <f>B13</f>
@@ -1314,37 +1283,31 @@
       </c>
       <c r="X7" s="4"/>
       <c r="Y7" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="Z7" s="3">
         <v>800</v>
       </c>
       <c r="AB7" s="4"/>
       <c r="AC7" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AD7" s="15">
+        <v>78</v>
+      </c>
+      <c r="AD7" s="18">
         <v>1580</v>
       </c>
       <c r="AE7" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AF7" s="10"/>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B8" s="3">
         <v>3000</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E8" s="3">
-        <v>531</v>
-      </c>
       <c r="I8" s="4"/>
       <c r="J8" s="3" t="s">
         <v>1</v>
@@ -1364,15 +1327,9 @@
         <v>287.5</v>
       </c>
       <c r="R8" s="4"/>
-      <c r="S8" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="T8" s="3">
-        <v>101</v>
-      </c>
       <c r="U8" s="4"/>
       <c r="V8" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="W8" s="3">
         <f>الأرصدة!L3</f>
@@ -1380,36 +1337,31 @@
       </c>
       <c r="X8" s="4"/>
       <c r="Y8" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="Z8" s="3">
         <v>1500</v>
       </c>
+      <c r="AA8" s="18"/>
       <c r="AB8" s="4"/>
       <c r="AC8" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="AD8" s="15">
+        <v>81</v>
+      </c>
+      <c r="AD8" s="18">
         <v>350</v>
       </c>
       <c r="AE8" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B9" s="3">
         <v>1500</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="F9" s="3">
-        <v>300</v>
-      </c>
       <c r="I9" s="4"/>
       <c r="J9" s="3" t="s">
         <v>3</v>
@@ -1421,29 +1373,23 @@
         <v>115</v>
       </c>
       <c r="O9" s="3">
-        <f t="shared" ref="O9:O24" si="0">SUM(K9:N9)</f>
+        <f t="shared" ref="O9:O17" si="0">SUM(K9:N9)</f>
         <v>195</v>
       </c>
       <c r="R9" s="4"/>
-      <c r="S9" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="T9" s="3">
-        <v>430</v>
-      </c>
       <c r="U9" s="4"/>
       <c r="V9" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="W9" s="3">
         <f>H5</f>
-        <v>787</v>
+        <v>7027</v>
       </c>
       <c r="X9" s="4"/>
       <c r="Y9" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="AA9" s="15">
+        <v>72</v>
+      </c>
+      <c r="AA9" s="20">
         <f>SUM(Z7:Z8)</f>
         <v>2300</v>
       </c>
@@ -1451,27 +1397,21 @@
       <c r="AC9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="AD9" s="15">
+      <c r="AD9" s="18">
         <v>80</v>
       </c>
       <c r="AE9" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B10" s="3">
         <v>2000</v>
       </c>
       <c r="C10" s="4"/>
-      <c r="D10" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="F10" s="3">
-        <v>1800</v>
-      </c>
       <c r="I10" s="4"/>
       <c r="J10" s="3" t="s">
         <v>4</v>
@@ -1486,37 +1426,32 @@
       <c r="R10" s="4"/>
       <c r="U10" s="4"/>
       <c r="V10" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="W10" s="3">
         <v>0</v>
       </c>
       <c r="X10" s="4"/>
+      <c r="AA10" s="18"/>
       <c r="AB10" s="4"/>
       <c r="AC10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AD10" s="15">
+      <c r="AD10" s="18">
         <v>80</v>
       </c>
       <c r="AE10" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B11" s="3">
         <v>5600</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="F11" s="3">
-        <v>300</v>
-      </c>
       <c r="I11" s="4"/>
       <c r="J11" s="3" t="s">
         <v>5</v>
@@ -1534,43 +1469,38 @@
         <v>55</v>
       </c>
       <c r="W11" s="3">
-        <v>27</v>
+        <f>J32</f>
+        <v>10077</v>
       </c>
       <c r="X11" s="4"/>
       <c r="Y11" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AA11" s="15">
+        <v>63</v>
+      </c>
+      <c r="AA11" s="20">
         <v>3000</v>
       </c>
       <c r="AB11" s="4"/>
       <c r="AC11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="AD11" s="15">
+        <v>73</v>
+      </c>
+      <c r="AD11" s="18">
         <v>120</v>
       </c>
       <c r="AE11" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B12" s="3">
         <v>1000</v>
       </c>
       <c r="C12" s="4"/>
-      <c r="D12" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="E12" s="3">
-        <v>276</v>
-      </c>
       <c r="I12" s="4"/>
       <c r="J12" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K12" s="3">
         <v>120</v>
@@ -1581,23 +1511,17 @@
       </c>
       <c r="R12" s="4"/>
       <c r="U12" s="4"/>
-      <c r="V12" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="W12" s="3">
-        <f>J32</f>
-        <v>3834</v>
-      </c>
       <c r="X12" s="4"/>
+      <c r="AA12" s="18"/>
       <c r="AB12" s="4"/>
       <c r="AC12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="AD12" s="3">
+      <c r="AD12" s="18">
         <v>77</v>
       </c>
       <c r="AE12" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.3">
@@ -1608,12 +1532,6 @@
         <v>3050</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="F13" s="3">
-        <v>345</v>
-      </c>
       <c r="I13" s="4"/>
       <c r="J13" s="3" t="s">
         <v>6</v>
@@ -1629,36 +1547,30 @@
       <c r="U13" s="4"/>
       <c r="X13" s="4"/>
       <c r="Y13" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA13" s="15">
+        <v>68</v>
+      </c>
+      <c r="AA13" s="20">
         <v>1000</v>
       </c>
       <c r="AB13" s="4"/>
       <c r="AC13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="AD13" s="3">
+      <c r="AD13" s="18">
         <v>150</v>
       </c>
       <c r="AE13" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B14" s="3">
         <v>1000</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="F14" s="3">
-        <v>300</v>
-      </c>
       <c r="I14" s="4"/>
       <c r="J14" s="3" t="s">
         <v>7</v>
@@ -1673,31 +1585,26 @@
       <c r="R14" s="4"/>
       <c r="U14" s="4"/>
       <c r="X14" s="4"/>
+      <c r="AA14" s="18"/>
       <c r="AB14" s="4"/>
       <c r="AC14" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="AD14" s="15">
+        <v>108</v>
+      </c>
+      <c r="AD14" s="18">
         <v>154</v>
       </c>
       <c r="AE14" s="3" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B15" s="3">
         <v>9027</v>
       </c>
       <c r="C15" s="4"/>
-      <c r="D15" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="F15" s="3">
-        <v>300</v>
-      </c>
       <c r="I15" s="4"/>
       <c r="J15" s="3" t="s">
         <v>8</v>
@@ -1713,31 +1620,26 @@
       <c r="U15" s="4"/>
       <c r="X15" s="4"/>
       <c r="Y15" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="Z15" s="3">
         <f>K27</f>
         <v>2345</v>
       </c>
+      <c r="AA15" s="18"/>
       <c r="AB15" s="4"/>
       <c r="AC15" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="AD15" s="15">
+        <v>111</v>
+      </c>
+      <c r="AD15" s="18">
         <v>301</v>
       </c>
       <c r="AE15" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.3">
       <c r="C16" s="4"/>
-      <c r="D16" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="F16" s="3">
-        <v>350</v>
-      </c>
       <c r="I16" s="4"/>
       <c r="J16" s="3" t="s">
         <v>9</v>
@@ -1753,150 +1655,139 @@
       <c r="U16" s="4"/>
       <c r="X16" s="4"/>
       <c r="Y16" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Z16" s="3">
         <v>1000</v>
       </c>
+      <c r="AA16" s="18"/>
       <c r="AB16" s="4"/>
     </row>
     <row r="17" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C17" s="4"/>
-      <c r="D17" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17" s="3">
-        <v>1200</v>
-      </c>
       <c r="I17" s="4"/>
-      <c r="J17" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="N17" s="3">
-        <v>27</v>
+      <c r="J17" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="K17" s="3">
+        <v>77</v>
       </c>
       <c r="O17" s="3">
-        <f t="shared" si="0"/>
-        <v>27</v>
+        <f>SUM(K17:N17)</f>
+        <v>77</v>
       </c>
       <c r="R17" s="4"/>
       <c r="U17" s="4"/>
       <c r="X17" s="4"/>
       <c r="Y17" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Z17" s="3">
         <v>0</v>
       </c>
+      <c r="AA17" s="18"/>
       <c r="AB17" s="4"/>
     </row>
     <row r="18" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C18" s="4"/>
-      <c r="D18" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="F18" s="3">
-        <v>350</v>
-      </c>
       <c r="I18" s="4"/>
-      <c r="J18" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="K18" s="3">
-        <v>77</v>
+      <c r="J18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L18" s="3">
+        <v>300</v>
       </c>
       <c r="O18" s="3">
-        <f t="shared" si="0"/>
-        <v>77</v>
+        <f>SUM(K18:N18)</f>
+        <v>300</v>
       </c>
       <c r="R18" s="4"/>
       <c r="U18" s="4"/>
       <c r="X18" s="4"/>
       <c r="Y18" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="Z18" s="3">
         <v>-150</v>
       </c>
+      <c r="AA18" s="18"/>
       <c r="AB18" s="4"/>
     </row>
     <row r="19" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L19" s="3">
-        <v>300</v>
+        <v>13</v>
+      </c>
+      <c r="K19" s="3">
+        <v>200</v>
       </c>
       <c r="O19" s="3">
-        <f t="shared" si="0"/>
-        <v>300</v>
+        <f>SUM(K19:N19)</f>
+        <v>200</v>
       </c>
       <c r="R19" s="4"/>
       <c r="U19" s="4"/>
       <c r="X19" s="4"/>
       <c r="Y19" s="3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="Z19" s="3">
-        <v>-77</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="AA19" s="18"/>
       <c r="AB19" s="4"/>
     </row>
     <row r="20" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C20" s="4"/>
       <c r="D20" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H20" s="3">
         <v>2000</v>
       </c>
       <c r="I20" s="4"/>
-      <c r="J20" s="3" t="s">
-        <v>13</v>
+      <c r="J20" s="14" t="s">
+        <v>14</v>
       </c>
       <c r="K20" s="3">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="O20" s="3">
-        <f t="shared" si="0"/>
-        <v>200</v>
+        <f>SUM(K20:N20)</f>
+        <v>150</v>
       </c>
       <c r="R20" s="4"/>
       <c r="U20" s="4"/>
       <c r="X20" s="4"/>
+      <c r="AA20" s="18"/>
       <c r="AB20" s="4"/>
     </row>
     <row r="21" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C21" s="4"/>
       <c r="D21" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="H21" s="3">
-        <f>T2</f>
-        <v>595</v>
+        <v>61</v>
       </c>
       <c r="I21" s="4"/>
-      <c r="J21" s="14" t="s">
-        <v>14</v>
+      <c r="J21" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="K21" s="3">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="O21" s="3">
-        <f t="shared" si="0"/>
-        <v>150</v>
+        <f>SUM(K21:N21)</f>
+        <v>0</v>
       </c>
       <c r="R21" s="4"/>
       <c r="U21" s="4"/>
       <c r="X21" s="4"/>
       <c r="Y21" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA21" s="15">
+        <v>79</v>
+      </c>
+      <c r="AA21" s="20">
         <f>SUM(Z15:Z20)</f>
-        <v>3118</v>
+        <v>3272</v>
       </c>
       <c r="AB21" s="4"/>
     </row>
@@ -1904,40 +1795,45 @@
       <c r="C22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K22" s="3">
+        <v>16</v>
+      </c>
+      <c r="M22" s="3">
         <v>0</v>
       </c>
       <c r="O22" s="3">
-        <f t="shared" si="0"/>
+        <f>SUM(K22:N22)</f>
         <v>0</v>
       </c>
       <c r="R22" s="4"/>
       <c r="U22" s="4"/>
       <c r="X22" s="4"/>
+      <c r="AA22" s="18"/>
       <c r="AB22" s="4"/>
     </row>
     <row r="23" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="3" t="s">
-        <v>16</v>
+        <v>131</v>
+      </c>
+      <c r="K23" s="22">
+        <f>(الأرصدة!AA2)-1667</f>
+        <v>1258</v>
       </c>
       <c r="M23" s="3">
-        <v>0</v>
+        <v>1667</v>
       </c>
       <c r="O23" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(K23:N23)</f>
+        <v>2925</v>
       </c>
       <c r="R23" s="4"/>
       <c r="U23" s="4"/>
       <c r="X23" s="4"/>
       <c r="Y23" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA23" s="15">
+        <v>80</v>
+      </c>
+      <c r="AA23" s="18">
         <f>L27</f>
         <v>820</v>
       </c>
@@ -1946,20 +1842,10 @@
     <row r="24" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="K24" s="3">
-        <f>الأرصدة!AA2</f>
-        <v>1258</v>
-      </c>
-      <c r="O24" s="3">
-        <f t="shared" si="0"/>
-        <v>1258</v>
-      </c>
       <c r="R24" s="4"/>
       <c r="U24" s="4"/>
       <c r="X24" s="4"/>
+      <c r="AA24" s="18"/>
       <c r="AB24" s="4"/>
     </row>
     <row r="25" spans="3:28" x14ac:dyDescent="0.3">
@@ -1969,9 +1855,9 @@
       <c r="U25" s="4"/>
       <c r="X25" s="4"/>
       <c r="Y25" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="AA25" s="15">
+        <v>90</v>
+      </c>
+      <c r="AA25" s="20">
         <v>2000</v>
       </c>
       <c r="AB25" s="4"/>
@@ -1982,6 +1868,7 @@
       <c r="R26" s="3"/>
       <c r="U26" s="3"/>
       <c r="X26" s="3"/>
+      <c r="AA26" s="18"/>
       <c r="AB26" s="3"/>
     </row>
     <row r="27" spans="3:28" x14ac:dyDescent="0.3">
@@ -2000,21 +1887,21 @@
       </c>
       <c r="M27" s="3">
         <f>SUM(M7:M25)</f>
-        <v>824</v>
+        <v>2752</v>
       </c>
       <c r="N27" s="3">
         <f>SUM(N7:N25)</f>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="R27" s="3"/>
       <c r="U27" s="3"/>
       <c r="X27" s="3"/>
       <c r="Y27" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA27" s="16">
+        <v>91</v>
+      </c>
+      <c r="AA27" s="19">
         <f>T2</f>
-        <v>595</v>
+        <v>0</v>
       </c>
       <c r="AB27" s="3"/>
     </row>
@@ -2024,6 +1911,7 @@
       <c r="R28" s="3"/>
       <c r="U28" s="3"/>
       <c r="X28" s="3"/>
+      <c r="AA28" s="18"/>
       <c r="AB28" s="3"/>
     </row>
     <row r="29" spans="3:28" x14ac:dyDescent="0.3">
@@ -2033,11 +1921,11 @@
       <c r="U29" s="3"/>
       <c r="X29" s="3"/>
       <c r="Y29" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA29" s="17">
+        <v>92</v>
+      </c>
+      <c r="AA29" s="21">
         <f>M27</f>
-        <v>824</v>
+        <v>2752</v>
       </c>
       <c r="AB29" s="3"/>
     </row>
@@ -2052,20 +1940,20 @@
     <row r="31" spans="3:28" ht="46" x14ac:dyDescent="0.3">
       <c r="C31" s="3"/>
       <c r="D31" s="13" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3" t="s">
         <v>19</v>
       </c>
       <c r="O31" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="P31" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="P31" s="3" t="s">
-        <v>60</v>
       </c>
       <c r="Q31" s="3" t="s">
         <v>20</v>
@@ -2074,18 +1962,18 @@
       <c r="U31" s="3"/>
       <c r="X31" s="3"/>
       <c r="Y31" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AA31" s="3">
+        <v>94</v>
+      </c>
+      <c r="AA31" s="20">
         <f>W2</f>
-        <v>7698</v>
+        <v>20154</v>
       </c>
       <c r="AB31" s="3"/>
     </row>
     <row r="32" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C32" s="3"/>
       <c r="D32">
-        <v>20221</v>
+        <v>21404</v>
       </c>
       <c r="E32" s="3" t="e">
         <f>D32+#REF!</f>
@@ -2094,19 +1982,19 @@
       <c r="I32" s="3"/>
       <c r="J32" s="3">
         <f>الأرصدة!M29-'مصاريف الشهر'!D32</f>
-        <v>3834</v>
+        <v>10077</v>
       </c>
       <c r="O32" s="3">
         <f>E3</f>
-        <v>2007</v>
+        <v>0</v>
       </c>
       <c r="P32" s="3">
         <f>F3</f>
-        <v>5645</v>
+        <v>0</v>
       </c>
       <c r="Q32" s="3">
         <f>J32-SUM(O32:P32)</f>
-        <v>-3818</v>
+        <v>10077</v>
       </c>
       <c r="R32" s="3"/>
       <c r="U32" s="3"/>
@@ -2115,12 +2003,12 @@
     </row>
     <row r="33" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y33" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y34" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="Z34" s="3">
         <v>0</v>
@@ -2133,51 +2021,45 @@
       </c>
     </row>
     <row r="36" spans="3:28" x14ac:dyDescent="0.3">
-      <c r="Y36" s="4"/>
-      <c r="Z36" s="4"/>
-      <c r="AA36" s="4"/>
+      <c r="Y36" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="AA36" s="3">
+        <v>1667</v>
+      </c>
     </row>
     <row r="37" spans="3:28" x14ac:dyDescent="0.3">
-      <c r="Y37" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="Z37" s="3">
-        <v>150</v>
-      </c>
+      <c r="Y37" s="4"/>
+      <c r="Z37" s="4"/>
+      <c r="AA37" s="4"/>
     </row>
     <row r="38" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y38" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="Z38" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39" spans="3:28" x14ac:dyDescent="0.3">
+      <c r="Y39" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="Z38" s="3">
+      <c r="Z39" s="3">
         <v>77</v>
       </c>
     </row>
-    <row r="39" spans="3:28" ht="46" x14ac:dyDescent="0.3">
-      <c r="Y39" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA39" s="3">
-        <f>SUM(Z37:Z38)</f>
+    <row r="40" spans="3:28" ht="46" x14ac:dyDescent="0.3">
+      <c r="Y40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="AA40" s="3">
+        <f>SUM(Z38:Z39)</f>
         <v>227</v>
       </c>
     </row>
-    <row r="40" spans="3:28" x14ac:dyDescent="0.3">
-      <c r="Y40" s="13"/>
-    </row>
     <row r="41" spans="3:28" x14ac:dyDescent="0.3">
-      <c r="C41" s="3"/>
-      <c r="I41" s="3"/>
-      <c r="R41" s="3"/>
-      <c r="U41" s="3"/>
-      <c r="X41" s="3"/>
-      <c r="Y41" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z41" s="3">
-        <v>2000</v>
-      </c>
-      <c r="AB41" s="3"/>
+      <c r="Y41" s="13"/>
     </row>
     <row r="42" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C42" s="3"/>
@@ -2186,11 +2068,10 @@
       <c r="U42" s="3"/>
       <c r="X42" s="3"/>
       <c r="Y42" s="3" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="Z42" s="3">
-        <f>G5</f>
-        <v>-423</v>
+        <v>2000</v>
       </c>
       <c r="AB42" s="3"/>
     </row>
@@ -2201,11 +2082,11 @@
       <c r="U43" s="3"/>
       <c r="X43" s="3"/>
       <c r="Y43" s="3" t="s">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="Z43" s="3">
-        <f>-Z17</f>
-        <v>0</v>
+        <f>G5</f>
+        <v>-317</v>
       </c>
       <c r="AB43" s="3"/>
     </row>
@@ -2216,21 +2097,35 @@
       <c r="U44" s="3"/>
       <c r="X44" s="3"/>
       <c r="Y44" s="3" t="s">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="Z44" s="3">
-        <f>AA39</f>
+        <v>-200</v>
+      </c>
+      <c r="AB44" s="3"/>
+    </row>
+    <row r="45" spans="3:28" x14ac:dyDescent="0.3">
+      <c r="C45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="R45" s="3"/>
+      <c r="U45" s="3"/>
+      <c r="X45" s="3"/>
+      <c r="Y45" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z45" s="3">
+        <f>AA40</f>
         <v>227</v>
       </c>
-      <c r="AB44" s="3"/>
-    </row>
-    <row r="45" spans="3:28" x14ac:dyDescent="0.3">
-      <c r="Y45" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA45" s="3">
-        <f>SUM(Z41:Z44)</f>
-        <v>1804</v>
+      <c r="AB45" s="3"/>
+    </row>
+    <row r="46" spans="3:28" x14ac:dyDescent="0.3">
+      <c r="Y46" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA46" s="3">
+        <f>SUM(Z42:Z45)</f>
+        <v>1710</v>
       </c>
     </row>
   </sheetData>
@@ -2254,7 +2149,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F05345A-5E98-0C43-BBDD-1D2CC38375ED}">
-  <dimension ref="A1:AG31"/>
+  <dimension ref="A1:AH31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -2284,16 +2179,18 @@
     <col min="25" max="25" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="0.5" customWidth="1"/>
     <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="20" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="0.5" customWidth="1"/>
+    <col min="28" max="28" width="20" customWidth="1"/>
+    <col min="29" max="29" width="8" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="0.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3" t="s">
@@ -2329,38 +2226,38 @@
       <c r="U1" s="3"/>
       <c r="V1" s="2"/>
       <c r="W1" s="3" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="Z1" s="4"/>
       <c r="AA1" s="3" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="AB1" s="3"/>
-      <c r="AC1" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="AD1" s="3" t="s">
-        <v>152</v>
+        <v>49</v>
       </c>
       <c r="AE1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="AF1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="AF1" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="AG1" s="4"/>
-    </row>
-    <row r="2" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AG1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH1" s="4"/>
+    </row>
+    <row r="2" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="11">
         <f>SUM(D6:D19)</f>
-        <v>10700</v>
+        <v>13750</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
@@ -2381,55 +2278,56 @@
       <c r="N2" s="4"/>
       <c r="O2" s="11">
         <f>SUM(Q6:Q20)</f>
-        <v>63052</v>
+        <v>70079</v>
       </c>
       <c r="P2" s="11"/>
       <c r="R2" s="4"/>
       <c r="S2" s="11">
         <f>SUM(U6:U19)</f>
-        <v>36405</v>
+        <v>39056</v>
       </c>
       <c r="T2" s="11"/>
       <c r="V2" s="2"/>
       <c r="W2" s="11">
-        <f>SUM(Y6:Y20)</f>
-        <v>9182</v>
+        <f>SUM(Y6:Y23)</f>
+        <v>11833</v>
       </c>
       <c r="X2" s="11">
-        <f>1500+(303*3)</f>
-        <v>2409</v>
+        <f>(1500+(303*3))+5001</f>
+        <v>7410</v>
       </c>
       <c r="Y2" s="11">
         <f>SUM(W2:X2)</f>
-        <v>11591</v>
+        <v>19243</v>
       </c>
       <c r="Z2" s="4"/>
       <c r="AA2" s="11">
-        <f>SUM(AF6:AF20)</f>
-        <v>1258</v>
+        <f>SUM(AG6:AG20)</f>
+        <v>2925</v>
       </c>
       <c r="AB2" s="11"/>
-      <c r="AC2" s="3">
-        <f>SUM(AC6:AC20)</f>
-        <v>4729</v>
-      </c>
+      <c r="AC2" s="11"/>
       <c r="AD2" s="3">
         <f>SUM(AD6:AD20)</f>
-        <v>1712</v>
+        <v>9730</v>
       </c>
       <c r="AE2" s="3">
         <f>SUM(AE6:AE20)</f>
-        <v>3017</v>
+        <v>1712</v>
       </c>
       <c r="AF2" s="3">
         <f>SUM(AF6:AF20)</f>
-        <v>1258</v>
-      </c>
-      <c r="AG2" s="4"/>
-    </row>
-    <row r="3" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+        <v>8018</v>
+      </c>
+      <c r="AG2" s="3">
+        <f>SUM(AG6:AG20)</f>
+        <v>2925</v>
+      </c>
+      <c r="AH2" s="4"/>
+    </row>
+    <row r="3" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="11">
@@ -2468,9 +2366,10 @@
       <c r="AD3" s="3"/>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
-      <c r="AG3" s="4"/>
-    </row>
-    <row r="4" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AG3" s="3"/>
+      <c r="AH3" s="4"/>
+    </row>
+    <row r="4" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B4" s="2"/>
       <c r="C4" s="3" t="s">
         <v>25</v>
@@ -2506,9 +2405,10 @@
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="3"/>
-      <c r="AG4" s="4"/>
-    </row>
-    <row r="5" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="4"/>
+    </row>
+    <row r="5" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="11"/>
@@ -2535,18 +2435,21 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="4"/>
       <c r="AA5" s="3" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="AB5" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="AC5" s="3"/>
+        <v>132</v>
+      </c>
+      <c r="AC5" s="3" t="s">
+        <v>140</v>
+      </c>
       <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
       <c r="AF5" s="3"/>
-      <c r="AG5" s="4"/>
-    </row>
-    <row r="6" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AG5" s="3"/>
+      <c r="AH5" s="4"/>
+    </row>
+    <row r="6" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
       <c r="C6" s="3" t="s">
         <v>26</v>
@@ -2600,7 +2503,7 @@
         <v>4</v>
       </c>
       <c r="X6" s="3" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="Y6" s="11">
         <v>200</v>
@@ -2610,24 +2513,27 @@
         <v>3</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AC6" s="3">
+        <v>136</v>
+      </c>
+      <c r="AC6" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AD6" s="3">
         <v>902</v>
       </c>
-      <c r="AD6" s="3">
+      <c r="AE6" s="3">
         <v>601</v>
       </c>
-      <c r="AE6" s="3">
-        <f>AC6-AD6</f>
+      <c r="AF6" s="3">
+        <f>AD6-AE6</f>
         <v>301</v>
       </c>
-      <c r="AF6" s="11">
+      <c r="AG6" s="11">
         <v>301</v>
       </c>
-      <c r="AG6" s="4"/>
-    </row>
-    <row r="7" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AH6" s="4"/>
+    </row>
+    <row r="7" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="3">
         <v>1</v>
@@ -2659,7 +2565,7 @@
         <v>1</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q7" s="11">
         <v>864</v>
@@ -2679,7 +2585,7 @@
         <v>4</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="Y7" s="11">
         <v>500</v>
@@ -2689,24 +2595,27 @@
         <v>4</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AC7" s="3">
+        <v>137</v>
+      </c>
+      <c r="AC7" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AD7" s="3">
         <v>1995</v>
       </c>
-      <c r="AD7" s="3">
+      <c r="AE7" s="3">
         <v>499</v>
       </c>
-      <c r="AE7" s="3">
-        <f>AC7-AD7</f>
+      <c r="AF7" s="3">
+        <f>AD7-AE7</f>
         <v>1496</v>
       </c>
-      <c r="AF7" s="3">
+      <c r="AG7" s="3">
         <v>499</v>
       </c>
-      <c r="AG7" s="4"/>
-    </row>
-    <row r="8" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AH7" s="4"/>
+    </row>
+    <row r="8" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
       <c r="C8" s="3">
         <v>1</v>
@@ -2740,7 +2649,7 @@
         <v>1</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="Q8" s="11">
         <v>17777</v>
@@ -2760,7 +2669,7 @@
         <v>4</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="Y8" s="11">
         <v>303</v>
@@ -2770,24 +2679,27 @@
         <v>4</v>
       </c>
       <c r="AB8" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="AC8" s="3">
+        <v>108</v>
+      </c>
+      <c r="AC8" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AD8" s="3">
         <v>616</v>
       </c>
-      <c r="AD8" s="3">
+      <c r="AE8" s="3">
         <v>308</v>
       </c>
-      <c r="AE8" s="3">
-        <f>AC8-AD8</f>
+      <c r="AF8" s="3">
+        <f>AD8-AE8</f>
         <v>308</v>
       </c>
-      <c r="AF8" s="11">
+      <c r="AG8" s="11">
         <v>154</v>
       </c>
-      <c r="AG8" s="4"/>
-    </row>
-    <row r="9" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AH8" s="4"/>
+    </row>
+    <row r="9" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
       <c r="C9" s="3">
         <v>2</v>
@@ -2821,7 +2733,7 @@
         <v>2</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q9" s="11">
         <v>1676</v>
@@ -2841,7 +2753,7 @@
         <v>4</v>
       </c>
       <c r="X9" s="3" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="Y9" s="11">
         <v>750</v>
@@ -2851,24 +2763,27 @@
         <v>4</v>
       </c>
       <c r="AB9" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="AC9" s="3">
+        <v>138</v>
+      </c>
+      <c r="AC9" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AD9" s="3">
         <v>1216</v>
       </c>
-      <c r="AD9" s="3">
+      <c r="AE9" s="3">
         <v>304</v>
       </c>
-      <c r="AE9" s="3">
-        <f>AC9-AD9</f>
+      <c r="AF9" s="3">
+        <f>AD9-AE9</f>
         <v>912</v>
       </c>
-      <c r="AF9" s="11">
+      <c r="AG9" s="11">
         <v>304</v>
       </c>
-      <c r="AG9" s="4"/>
-    </row>
-    <row r="10" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AH9" s="4"/>
+    </row>
+    <row r="10" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
       <c r="C10" s="3">
         <v>3</v>
@@ -2896,7 +2811,7 @@
         <v>3</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q10" s="11">
         <v>787</v>
@@ -2916,26 +2831,46 @@
         <v>4</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="Y10" s="11">
         <v>188</v>
       </c>
       <c r="Z10" s="4"/>
-      <c r="AA10" s="3"/>
-      <c r="AB10" s="3"/>
-      <c r="AC10" s="3"/>
-      <c r="AD10" s="3"/>
-      <c r="AE10" s="3"/>
-      <c r="AF10" s="11"/>
-      <c r="AG10" s="4"/>
-    </row>
-    <row r="11" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AA10" s="3">
+        <v>4</v>
+      </c>
+      <c r="AB10" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="AC10" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD10" s="15">
+        <f>AG10*3</f>
+        <v>5001</v>
+      </c>
+      <c r="AE10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="3">
+        <f>AD10-AE10</f>
+        <v>5001</v>
+      </c>
+      <c r="AG10" s="11">
+        <f>1618+49</f>
+        <v>1667</v>
+      </c>
+      <c r="AH10" s="4"/>
+    </row>
+    <row r="11" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
       <c r="C11" s="3">
         <v>4</v>
       </c>
-      <c r="D11" s="11"/>
+      <c r="D11" s="11">
+        <v>3050</v>
+      </c>
       <c r="E11" s="4"/>
       <c r="F11" s="3">
         <v>5</v>
@@ -2954,7 +2889,7 @@
         <v>4</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="Q11" s="11">
         <v>2000</v>
@@ -2974,7 +2909,7 @@
         <v>4</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="Y11" s="11">
         <v>200</v>
@@ -2985,10 +2920,11 @@
       <c r="AC11" s="3"/>
       <c r="AD11" s="3"/>
       <c r="AE11" s="3"/>
-      <c r="AF11" s="11"/>
-      <c r="AG11" s="4"/>
-    </row>
-    <row r="12" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF11" s="3"/>
+      <c r="AG11" s="11"/>
+      <c r="AH11" s="4"/>
+    </row>
+    <row r="12" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="3">
         <v>5</v>
@@ -3008,15 +2944,21 @@
       </c>
       <c r="M12" s="11"/>
       <c r="N12" s="4"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="11"/>
+      <c r="O12" s="3">
+        <v>4</v>
+      </c>
+      <c r="P12" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q12" s="11">
+        <v>7027</v>
+      </c>
       <c r="R12" s="4"/>
       <c r="S12">
         <v>2</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="U12" s="11">
         <v>10000</v>
@@ -3026,7 +2968,7 @@
         <v>4</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="Y12" s="11">
         <v>200</v>
@@ -3037,10 +2979,11 @@
       <c r="AC12" s="3"/>
       <c r="AD12" s="3"/>
       <c r="AE12" s="3"/>
-      <c r="AF12" s="11"/>
-      <c r="AG12" s="4"/>
-    </row>
-    <row r="13" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF12" s="3"/>
+      <c r="AG12" s="11"/>
+      <c r="AH12" s="4"/>
+    </row>
+    <row r="13" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="3">
         <v>6</v>
@@ -3068,7 +3011,7 @@
         <v>2</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="U13" s="11">
         <v>1000</v>
@@ -3078,7 +3021,7 @@
         <v>4</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="Y13" s="11">
         <v>223</v>
@@ -3089,10 +3032,11 @@
       <c r="AC13" s="3"/>
       <c r="AD13" s="3"/>
       <c r="AE13" s="3"/>
-      <c r="AF13" s="11"/>
-      <c r="AG13" s="4"/>
-    </row>
-    <row r="14" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF13" s="3"/>
+      <c r="AG13" s="11"/>
+      <c r="AH13" s="4"/>
+    </row>
+    <row r="14" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="3">
         <v>7</v>
@@ -3118,7 +3062,7 @@
         <v>2</v>
       </c>
       <c r="T14" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="U14" s="11">
         <v>500</v>
@@ -3128,7 +3072,7 @@
         <v>4</v>
       </c>
       <c r="X14" s="3" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="Y14" s="11">
         <v>1883</v>
@@ -3139,10 +3083,11 @@
       <c r="AC14" s="3"/>
       <c r="AD14" s="3"/>
       <c r="AE14" s="3"/>
-      <c r="AF14" s="11"/>
-      <c r="AG14" s="4"/>
-    </row>
-    <row r="15" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="11"/>
+      <c r="AH14" s="4"/>
+    </row>
+    <row r="15" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="3">
         <v>8</v>
@@ -3168,7 +3113,7 @@
         <v>3</v>
       </c>
       <c r="T15" s="3" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="U15" s="3">
         <v>3701</v>
@@ -3178,7 +3123,7 @@
         <v>4</v>
       </c>
       <c r="X15" s="3" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="Y15" s="11">
         <v>501</v>
@@ -3189,10 +3134,11 @@
       <c r="AC15" s="3"/>
       <c r="AD15" s="3"/>
       <c r="AE15" s="3"/>
-      <c r="AF15" s="11"/>
-      <c r="AG15" s="4"/>
-    </row>
-    <row r="16" spans="1:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF15" s="3"/>
+      <c r="AG15" s="11"/>
+      <c r="AH15" s="4"/>
+    </row>
+    <row r="16" spans="1:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="3">
         <v>9</v>
@@ -3218,7 +3164,7 @@
         <v>3</v>
       </c>
       <c r="T16" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="U16" s="3">
         <v>1000</v>
@@ -3228,7 +3174,7 @@
         <v>4</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="Y16" s="11">
         <v>1500</v>
@@ -3239,10 +3185,11 @@
       <c r="AC16" s="3"/>
       <c r="AD16" s="3"/>
       <c r="AE16" s="3"/>
-      <c r="AF16" s="11"/>
-      <c r="AG16" s="4"/>
-    </row>
-    <row r="17" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="11"/>
+      <c r="AH16" s="4"/>
+    </row>
+    <row r="17" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
       <c r="C17" s="3">
         <v>10</v>
@@ -3268,7 +3215,7 @@
         <v>3</v>
       </c>
       <c r="T17" s="3" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="U17" s="11">
         <v>850</v>
@@ -3278,7 +3225,7 @@
         <v>4</v>
       </c>
       <c r="X17" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="Y17" s="11"/>
       <c r="Z17" s="4"/>
@@ -3287,10 +3234,11 @@
       <c r="AC17" s="3"/>
       <c r="AD17" s="3"/>
       <c r="AE17" s="3"/>
-      <c r="AF17" s="11"/>
-      <c r="AG17" s="4"/>
-    </row>
-    <row r="18" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF17" s="3"/>
+      <c r="AG17" s="11"/>
+      <c r="AH17" s="4"/>
+    </row>
+    <row r="18" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
       <c r="C18" s="3">
         <v>11</v>
@@ -3315,20 +3263,20 @@
       <c r="S18" s="3">
         <v>4</v>
       </c>
-      <c r="T18" s="18" t="str">
+      <c r="T18" s="15" t="str">
         <f>W1</f>
         <v>سفرة مصر</v>
       </c>
       <c r="U18" s="11">
         <f>W2</f>
-        <v>9182</v>
+        <v>11833</v>
       </c>
       <c r="V18" s="2"/>
       <c r="W18" s="3">
         <v>10</v>
       </c>
       <c r="X18" s="3" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="Y18" s="11">
         <v>2734</v>
@@ -3339,10 +3287,11 @@
       <c r="AC18" s="3"/>
       <c r="AD18" s="3"/>
       <c r="AE18" s="3"/>
-      <c r="AF18" s="11"/>
-      <c r="AG18" s="4"/>
-    </row>
-    <row r="19" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AF18" s="3"/>
+      <c r="AG18" s="11"/>
+      <c r="AH18" s="4"/>
+    </row>
+    <row r="19" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B19" s="2"/>
       <c r="C19" s="3">
         <v>12</v>
@@ -3366,9 +3315,15 @@
       <c r="T19" s="3"/>
       <c r="U19" s="11"/>
       <c r="V19" s="2"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
-      <c r="Y19" s="3"/>
+      <c r="W19" s="3">
+        <v>4</v>
+      </c>
+      <c r="X19" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="Y19" s="3">
+        <v>228</v>
+      </c>
       <c r="Z19" s="4"/>
       <c r="AA19" s="3"/>
       <c r="AB19" s="3"/>
@@ -3376,9 +3331,10 @@
       <c r="AD19" s="3"/>
       <c r="AE19" s="3"/>
       <c r="AF19" s="3"/>
-      <c r="AG19" s="4"/>
-    </row>
-    <row r="20" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AG19" s="3"/>
+      <c r="AH19" s="4"/>
+    </row>
+    <row r="20" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B20" s="2"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
@@ -3400,9 +3356,15 @@
       <c r="T20" s="3"/>
       <c r="U20" s="11"/>
       <c r="V20" s="2"/>
-      <c r="W20" s="3"/>
-      <c r="X20" s="3"/>
-      <c r="Y20" s="3"/>
+      <c r="W20" s="3">
+        <v>4</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="Y20" s="5">
+        <v>1957</v>
+      </c>
       <c r="Z20" s="4"/>
       <c r="AA20" s="3"/>
       <c r="AB20" s="3"/>
@@ -3410,9 +3372,10 @@
       <c r="AD20" s="3"/>
       <c r="AE20" s="3"/>
       <c r="AF20" s="3"/>
-      <c r="AG20" s="4"/>
-    </row>
-    <row r="21" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AG20" s="3"/>
+      <c r="AH20" s="4"/>
+    </row>
+    <row r="21" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="B21" s="2"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -3434,9 +3397,15 @@
       <c r="T21" s="4"/>
       <c r="U21" s="4"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="4"/>
-      <c r="X21" s="4"/>
-      <c r="Y21" s="4"/>
+      <c r="W21" s="3">
+        <v>4</v>
+      </c>
+      <c r="X21" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y21" s="11">
+        <v>466</v>
+      </c>
       <c r="Z21" s="4"/>
       <c r="AA21" s="4"/>
       <c r="AB21" s="4"/>
@@ -3445,8 +3414,9 @@
       <c r="AE21" s="4"/>
       <c r="AF21" s="4"/>
       <c r="AG21" s="4"/>
-    </row>
-    <row r="22" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="AH21" s="4"/>
+    </row>
+    <row r="22" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
@@ -3467,7 +3437,7 @@
       <c r="T22" s="3"/>
       <c r="U22" s="3"/>
     </row>
-    <row r="23" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
@@ -3482,7 +3452,7 @@
       </c>
       <c r="M23" s="6">
         <f>O2-S2</f>
-        <v>26647</v>
+        <v>31023</v>
       </c>
       <c r="N23" s="4"/>
       <c r="O23" s="3"/>
@@ -3493,7 +3463,7 @@
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
     </row>
-    <row r="24" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
@@ -3508,7 +3478,7 @@
       </c>
       <c r="M24" s="6">
         <f>C2</f>
-        <v>10700</v>
+        <v>13750</v>
       </c>
       <c r="N24" s="4"/>
       <c r="O24" s="3"/>
@@ -3518,8 +3488,11 @@
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
-    </row>
-    <row r="25" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+      <c r="W24" s="4"/>
+      <c r="X24" s="4"/>
+      <c r="Y24" s="4"/>
+    </row>
+    <row r="25" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
@@ -3545,7 +3518,7 @@
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
     </row>
-    <row r="26" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
@@ -3571,10 +3544,10 @@
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
       <c r="Y26" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="27" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
@@ -3585,7 +3558,7 @@
       <c r="J27" s="3"/>
       <c r="K27" s="4"/>
       <c r="L27" s="3" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="M27" s="6">
         <v>-10500</v>
@@ -3603,10 +3576,10 @@
       </c>
       <c r="Y27" s="12">
         <f>M29-W27</f>
-        <v>-11211</v>
-      </c>
-    </row>
-    <row r="28" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+        <v>-3785</v>
+      </c>
+    </row>
+    <row r="28" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
@@ -3632,7 +3605,7 @@
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
     </row>
-    <row r="29" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
@@ -3647,7 +3620,7 @@
       </c>
       <c r="M29" s="6">
         <f>SUM(M23:M28)</f>
-        <v>24055</v>
+        <v>31481</v>
       </c>
       <c r="N29" s="4"/>
       <c r="O29" s="3"/>
@@ -3658,7 +3631,7 @@
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
     </row>
-    <row r="30" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
@@ -3675,7 +3648,7 @@
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
     </row>
-    <row r="31" spans="2:33" ht="22" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>

</xml_diff>

<commit_message>
April 2026 - Finalized2
</commit_message>
<xml_diff>
--- a/April 2026.xlsx
+++ b/April 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abutalib/Projects/personal-accounting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A398737A-5BAB-C641-8DEB-C8865F9944DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5D7055F-CFFD-A24B-AC6D-B817BB5F91CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
   </bookViews>
   <sheets>
     <sheet name="مصاريف الشهر" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="148">
   <si>
     <t>فاتورة الكهرباء</t>
   </si>
@@ -423,9 +423,6 @@
     <t>حجز فندق ١ يوم</t>
   </si>
   <si>
-    <t>دولارات</t>
-  </si>
-  <si>
     <t>جنيهات</t>
   </si>
   <si>
@@ -477,13 +474,13 @@
     <t>رسوم الفحص</t>
   </si>
   <si>
-    <t>العملية  4,951  متوقع</t>
-  </si>
-  <si>
     <t>اسكندرية</t>
   </si>
   <si>
     <t>قسط الراجحي</t>
+  </si>
+  <si>
+    <t>العملية  4,951 تم تقسيطها</t>
   </si>
 </sst>
 </file>
@@ -603,7 +600,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -622,19 +619,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1037,14 +1033,14 @@
       <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17" t="s">
+      <c r="F1" s="21"/>
+      <c r="G1" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="17"/>
+      <c r="H1" s="21"/>
       <c r="I1" s="4"/>
       <c r="J1" s="3" t="s">
         <v>17</v>
@@ -1105,7 +1101,7 @@
       </c>
       <c r="W2" s="3">
         <f>SUM(W7:W16)</f>
-        <v>20154</v>
+        <v>22024</v>
       </c>
       <c r="X2" s="4"/>
       <c r="Y2" s="3" t="s">
@@ -1113,7 +1109,7 @@
       </c>
       <c r="AA2" s="3">
         <f>SUM(AA7:AB35)</f>
-        <v>35298</v>
+        <v>37168</v>
       </c>
       <c r="AB2" s="4"/>
       <c r="AC2" s="3" t="s">
@@ -1237,10 +1233,10 @@
       <c r="O6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P6" s="16" t="s">
+      <c r="P6" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="Q6" s="16"/>
+      <c r="Q6" s="20"/>
       <c r="R6" s="9"/>
       <c r="U6" s="9"/>
       <c r="X6" s="9"/>
@@ -1292,7 +1288,7 @@
       <c r="AC7" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="AD7" s="18">
+      <c r="AD7" s="3">
         <v>1580</v>
       </c>
       <c r="AE7" s="3" t="s">
@@ -1342,12 +1338,11 @@
       <c r="Z8" s="3">
         <v>1500</v>
       </c>
-      <c r="AA8" s="18"/>
       <c r="AB8" s="4"/>
       <c r="AC8" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="AD8" s="18">
+      <c r="AD8" s="3">
         <v>350</v>
       </c>
       <c r="AE8" s="3" t="s">
@@ -1373,7 +1368,7 @@
         <v>115</v>
       </c>
       <c r="O9" s="3">
-        <f t="shared" ref="O9:O17" si="0">SUM(K9:N9)</f>
+        <f t="shared" ref="O9:O16" si="0">SUM(K9:N9)</f>
         <v>195</v>
       </c>
       <c r="R9" s="4"/>
@@ -1389,7 +1384,7 @@
       <c r="Y9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AA9" s="20">
+      <c r="AA9" s="17">
         <f>SUM(Z7:Z8)</f>
         <v>2300</v>
       </c>
@@ -1397,7 +1392,7 @@
       <c r="AC9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="AD9" s="18">
+      <c r="AD9" s="3">
         <v>80</v>
       </c>
       <c r="AE9" s="3" t="s">
@@ -1432,12 +1427,11 @@
         <v>0</v>
       </c>
       <c r="X10" s="4"/>
-      <c r="AA10" s="18"/>
       <c r="AB10" s="4"/>
       <c r="AC10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AD10" s="18">
+      <c r="AD10" s="3">
         <v>80</v>
       </c>
       <c r="AE10" s="3" t="s">
@@ -1470,20 +1464,20 @@
       </c>
       <c r="W11" s="3">
         <f>J32</f>
-        <v>10077</v>
+        <v>11947</v>
       </c>
       <c r="X11" s="4"/>
       <c r="Y11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AA11" s="20">
+      <c r="AA11" s="17">
         <v>3000</v>
       </c>
       <c r="AB11" s="4"/>
       <c r="AC11" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AD11" s="18">
+      <c r="AD11" s="3">
         <v>120</v>
       </c>
       <c r="AE11" s="3" t="s">
@@ -1512,12 +1506,11 @@
       <c r="R12" s="4"/>
       <c r="U12" s="4"/>
       <c r="X12" s="4"/>
-      <c r="AA12" s="18"/>
       <c r="AB12" s="4"/>
       <c r="AC12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="AD12" s="18">
+      <c r="AD12" s="3">
         <v>77</v>
       </c>
       <c r="AE12" s="3" t="s">
@@ -1549,14 +1542,14 @@
       <c r="Y13" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AA13" s="20">
+      <c r="AA13" s="17">
         <v>1000</v>
       </c>
       <c r="AB13" s="4"/>
       <c r="AC13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="AD13" s="18">
+      <c r="AD13" s="3">
         <v>150</v>
       </c>
       <c r="AE13" s="3" t="s">
@@ -1585,12 +1578,11 @@
       <c r="R14" s="4"/>
       <c r="U14" s="4"/>
       <c r="X14" s="4"/>
-      <c r="AA14" s="18"/>
       <c r="AB14" s="4"/>
       <c r="AC14" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="AD14" s="18">
+      <c r="AD14" s="3">
         <v>154</v>
       </c>
       <c r="AE14" s="3" t="s">
@@ -1626,12 +1618,11 @@
         <f>K27</f>
         <v>2345</v>
       </c>
-      <c r="AA15" s="18"/>
       <c r="AB15" s="4"/>
       <c r="AC15" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="AD15" s="18">
+      <c r="AD15" s="3">
         <v>301</v>
       </c>
       <c r="AE15" s="3" t="s">
@@ -1660,7 +1651,6 @@
       <c r="Z16" s="3">
         <v>1000</v>
       </c>
-      <c r="AA16" s="18"/>
       <c r="AB16" s="4"/>
     </row>
     <row r="17" spans="3:28" x14ac:dyDescent="0.3">
@@ -1673,7 +1663,7 @@
         <v>77</v>
       </c>
       <c r="O17" s="3">
-        <f>SUM(K17:N17)</f>
+        <f t="shared" ref="O17:O23" si="1">SUM(K17:N17)</f>
         <v>77</v>
       </c>
       <c r="R17" s="4"/>
@@ -1685,7 +1675,6 @@
       <c r="Z17" s="3">
         <v>0</v>
       </c>
-      <c r="AA17" s="18"/>
       <c r="AB17" s="4"/>
     </row>
     <row r="18" spans="3:28" x14ac:dyDescent="0.3">
@@ -1698,7 +1687,7 @@
         <v>300</v>
       </c>
       <c r="O18" s="3">
-        <f>SUM(K18:N18)</f>
+        <f t="shared" si="1"/>
         <v>300</v>
       </c>
       <c r="R18" s="4"/>
@@ -1710,7 +1699,6 @@
       <c r="Z18" s="3">
         <v>-150</v>
       </c>
-      <c r="AA18" s="18"/>
       <c r="AB18" s="4"/>
     </row>
     <row r="19" spans="3:28" x14ac:dyDescent="0.3">
@@ -1723,7 +1711,7 @@
         <v>200</v>
       </c>
       <c r="O19" s="3">
-        <f>SUM(K19:N19)</f>
+        <f t="shared" si="1"/>
         <v>200</v>
       </c>
       <c r="R19" s="4"/>
@@ -1735,7 +1723,6 @@
       <c r="Z19" s="3">
         <v>77</v>
       </c>
-      <c r="AA19" s="18"/>
       <c r="AB19" s="4"/>
     </row>
     <row r="20" spans="3:28" x14ac:dyDescent="0.3">
@@ -1754,13 +1741,12 @@
         <v>150</v>
       </c>
       <c r="O20" s="3">
-        <f>SUM(K20:N20)</f>
+        <f t="shared" si="1"/>
         <v>150</v>
       </c>
       <c r="R20" s="4"/>
       <c r="U20" s="4"/>
       <c r="X20" s="4"/>
-      <c r="AA20" s="18"/>
       <c r="AB20" s="4"/>
     </row>
     <row r="21" spans="3:28" x14ac:dyDescent="0.3">
@@ -1776,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="3">
-        <f>SUM(K21:N21)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R21" s="4"/>
@@ -1785,7 +1771,7 @@
       <c r="Y21" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="AA21" s="20">
+      <c r="AA21" s="17">
         <f>SUM(Z15:Z20)</f>
         <v>3272</v>
       </c>
@@ -1801,22 +1787,21 @@
         <v>0</v>
       </c>
       <c r="O22" s="3">
-        <f>SUM(K22:N22)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R22" s="4"/>
       <c r="U22" s="4"/>
       <c r="X22" s="4"/>
-      <c r="AA22" s="18"/>
       <c r="AB22" s="4"/>
     </row>
     <row r="23" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="K23" s="22">
+        <v>130</v>
+      </c>
+      <c r="K23" s="19">
         <f>(الأرصدة!AA2)-1667</f>
         <v>1258</v>
       </c>
@@ -1824,7 +1809,7 @@
         <v>1667</v>
       </c>
       <c r="O23" s="3">
-        <f>SUM(K23:N23)</f>
+        <f t="shared" si="1"/>
         <v>2925</v>
       </c>
       <c r="R23" s="4"/>
@@ -1833,7 +1818,7 @@
       <c r="Y23" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="AA23" s="18">
+      <c r="AA23" s="3">
         <f>L27</f>
         <v>820</v>
       </c>
@@ -1845,7 +1830,6 @@
       <c r="R24" s="4"/>
       <c r="U24" s="4"/>
       <c r="X24" s="4"/>
-      <c r="AA24" s="18"/>
       <c r="AB24" s="4"/>
     </row>
     <row r="25" spans="3:28" x14ac:dyDescent="0.3">
@@ -1857,7 +1841,7 @@
       <c r="Y25" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="AA25" s="20">
+      <c r="AA25" s="17">
         <v>2000</v>
       </c>
       <c r="AB25" s="4"/>
@@ -1868,7 +1852,6 @@
       <c r="R26" s="3"/>
       <c r="U26" s="3"/>
       <c r="X26" s="3"/>
-      <c r="AA26" s="18"/>
       <c r="AB26" s="3"/>
     </row>
     <row r="27" spans="3:28" x14ac:dyDescent="0.3">
@@ -1899,7 +1882,7 @@
       <c r="Y27" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="AA27" s="19">
+      <c r="AA27" s="16">
         <f>T2</f>
         <v>0</v>
       </c>
@@ -1911,7 +1894,6 @@
       <c r="R28" s="3"/>
       <c r="U28" s="3"/>
       <c r="X28" s="3"/>
-      <c r="AA28" s="18"/>
       <c r="AB28" s="3"/>
     </row>
     <row r="29" spans="3:28" x14ac:dyDescent="0.3">
@@ -1923,7 +1905,7 @@
       <c r="Y29" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="AA29" s="21">
+      <c r="AA29" s="18">
         <f>M27</f>
         <v>2752</v>
       </c>
@@ -1964,9 +1946,9 @@
       <c r="Y31" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="AA31" s="20">
+      <c r="AA31" s="17">
         <f>W2</f>
-        <v>20154</v>
+        <v>22024</v>
       </c>
       <c r="AB31" s="3"/>
     </row>
@@ -1982,7 +1964,7 @@
       <c r="I32" s="3"/>
       <c r="J32" s="3">
         <f>الأرصدة!M29-'مصاريف الشهر'!D32</f>
-        <v>10077</v>
+        <v>11947</v>
       </c>
       <c r="O32" s="3">
         <f>E3</f>
@@ -1994,7 +1976,7 @@
       </c>
       <c r="Q32" s="3">
         <f>J32-SUM(O32:P32)</f>
-        <v>10077</v>
+        <v>11947</v>
       </c>
       <c r="R32" s="3"/>
       <c r="U32" s="3"/>
@@ -2022,7 +2004,7 @@
     </row>
     <row r="36" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y36" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="AA36" s="3">
         <v>1667</v>
@@ -2233,20 +2215,20 @@
       </c>
       <c r="Z1" s="4"/>
       <c r="AA1" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AB1" s="3"/>
       <c r="AD1" s="3" t="s">
         <v>49</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AF1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AH1" s="4"/>
     </row>
@@ -2284,13 +2266,13 @@
       <c r="R2" s="4"/>
       <c r="S2" s="11">
         <f>SUM(U6:U19)</f>
-        <v>39056</v>
+        <v>37186</v>
       </c>
       <c r="T2" s="11"/>
       <c r="V2" s="2"/>
       <c r="W2" s="11">
         <f>SUM(Y6:Y23)</f>
-        <v>11833</v>
+        <v>9963</v>
       </c>
       <c r="X2" s="11">
         <f>(1500+(303*3))+5001</f>
@@ -2298,7 +2280,7 @@
       </c>
       <c r="Y2" s="11">
         <f>SUM(W2:X2)</f>
-        <v>19243</v>
+        <v>17373</v>
       </c>
       <c r="Z2" s="4"/>
       <c r="AA2" s="11">
@@ -2435,13 +2417,13 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="4"/>
       <c r="AA5" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AB5" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AC5" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
@@ -2513,10 +2495,10 @@
         <v>3</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC6" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AD6" s="3">
         <v>902</v>
@@ -2595,10 +2577,10 @@
         <v>4</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AC7" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AD7" s="3">
         <v>1995</v>
@@ -2682,7 +2664,7 @@
         <v>108</v>
       </c>
       <c r="AC8" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AD8" s="3">
         <v>616</v>
@@ -2763,10 +2745,10 @@
         <v>4</v>
       </c>
       <c r="AB9" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AC9" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AD9" s="3">
         <v>1216</v>
@@ -2841,7 +2823,7 @@
         <v>4</v>
       </c>
       <c r="AB10" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AC10" s="3" t="s">
         <v>103</v>
@@ -3075,7 +3057,7 @@
         <v>128</v>
       </c>
       <c r="Y14" s="11">
-        <v>1883</v>
+        <v>501</v>
       </c>
       <c r="Z14" s="4"/>
       <c r="AA14" s="3"/>
@@ -3126,7 +3108,7 @@
         <v>129</v>
       </c>
       <c r="Y15" s="11">
-        <v>501</v>
+        <v>1500</v>
       </c>
       <c r="Z15" s="4"/>
       <c r="AA15" s="3"/>
@@ -3174,11 +3156,9 @@
         <v>4</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="Y16" s="11">
-        <v>1500</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="Y16" s="11"/>
       <c r="Z16" s="4"/>
       <c r="AA16" s="3"/>
       <c r="AB16" s="3"/>
@@ -3222,12 +3202,14 @@
       </c>
       <c r="V17" s="2"/>
       <c r="W17" s="3">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="X17" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="Y17" s="11"/>
+        <v>138</v>
+      </c>
+      <c r="Y17" s="11">
+        <v>2734</v>
+      </c>
       <c r="Z17" s="4"/>
       <c r="AA17" s="3"/>
       <c r="AB17" s="3"/>
@@ -3269,17 +3251,17 @@
       </c>
       <c r="U18" s="11">
         <f>W2</f>
-        <v>11833</v>
+        <v>9963</v>
       </c>
       <c r="V18" s="2"/>
       <c r="W18" s="3">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="X18" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="Y18" s="11">
-        <v>2734</v>
+        <v>142</v>
+      </c>
+      <c r="Y18" s="3">
+        <v>228</v>
       </c>
       <c r="Z18" s="4"/>
       <c r="AA18" s="3"/>
@@ -3321,8 +3303,8 @@
       <c r="X19" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="Y19" s="3">
-        <v>228</v>
+      <c r="Y19" s="5">
+        <v>1957</v>
       </c>
       <c r="Z19" s="4"/>
       <c r="AA19" s="3"/>
@@ -3360,10 +3342,10 @@
         <v>4</v>
       </c>
       <c r="X20" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="Y20" s="5">
-        <v>1957</v>
+        <v>145</v>
+      </c>
+      <c r="Y20" s="11">
+        <v>479</v>
       </c>
       <c r="Z20" s="4"/>
       <c r="AA20" s="3"/>
@@ -3397,15 +3379,6 @@
       <c r="T21" s="4"/>
       <c r="U21" s="4"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="3">
-        <v>4</v>
-      </c>
-      <c r="X21" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="Y21" s="11">
-        <v>466</v>
-      </c>
       <c r="Z21" s="4"/>
       <c r="AA21" s="4"/>
       <c r="AB21" s="4"/>
@@ -3452,7 +3425,7 @@
       </c>
       <c r="M23" s="6">
         <f>O2-S2</f>
-        <v>31023</v>
+        <v>32893</v>
       </c>
       <c r="N23" s="4"/>
       <c r="O23" s="3"/>
@@ -3576,7 +3549,7 @@
       </c>
       <c r="Y27" s="12">
         <f>M29-W27</f>
-        <v>-3785</v>
+        <v>-1915</v>
       </c>
     </row>
     <row r="28" spans="2:34" ht="22" x14ac:dyDescent="0.3">
@@ -3620,7 +3593,7 @@
       </c>
       <c r="M29" s="6">
         <f>SUM(M23:M28)</f>
-        <v>31481</v>
+        <v>33351</v>
       </c>
       <c r="N29" s="4"/>
       <c r="O29" s="3"/>

</xml_diff>

<commit_message>
April 2026 - Finalized3
</commit_message>
<xml_diff>
--- a/April 2026.xlsx
+++ b/April 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abutalib/Projects/personal-accounting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5D7055F-CFFD-A24B-AC6D-B817BB5F91CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359721AD-E0FB-6449-BB3C-0113D55D02AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{7E62CB60-3E82-0E48-87C0-051D0E492E72}"/>
   </bookViews>
   <sheets>
     <sheet name="مصاريف الشهر" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="148">
   <si>
     <t>فاتورة الكهرباء</t>
   </si>
@@ -303,9 +303,6 @@
     <t>digital ocean</t>
   </si>
   <si>
-    <t>month 1st</t>
-  </si>
-  <si>
     <t>month 5th</t>
   </si>
   <si>
@@ -417,9 +414,6 @@
     <t>غير معروف</t>
   </si>
   <si>
-    <t>دفعات متبقية</t>
-  </si>
-  <si>
     <t>حجز فندق ١ يوم</t>
   </si>
   <si>
@@ -481,6 +475,12 @@
   </si>
   <si>
     <t>العملية  4,951 تم تقسيطها</t>
+  </si>
+  <si>
+    <t>دفعات مقسطة</t>
+  </si>
+  <si>
+    <t>month 9st</t>
   </si>
 </sst>
 </file>
@@ -600,7 +600,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -618,7 +618,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
@@ -1033,14 +1032,14 @@
       <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21" t="s">
+      <c r="F1" s="20"/>
+      <c r="G1" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="21"/>
+      <c r="H1" s="20"/>
       <c r="I1" s="4"/>
       <c r="J1" s="3" t="s">
         <v>17</v>
@@ -1055,7 +1054,7 @@
       </c>
       <c r="X1" s="4"/>
       <c r="Y1" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AB1" s="4"/>
       <c r="AC1" s="3" t="s">
@@ -1225,7 +1224,7 @@
         <v>75</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="N6" s="8" t="s">
         <v>57</v>
@@ -1233,10 +1232,10 @@
       <c r="O6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P6" s="20" t="s">
+      <c r="P6" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="Q6" s="20"/>
+      <c r="Q6" s="19"/>
       <c r="R6" s="9"/>
       <c r="U6" s="9"/>
       <c r="X6" s="9"/>
@@ -1291,7 +1290,7 @@
       <c r="AD7" s="3">
         <v>1580</v>
       </c>
-      <c r="AE7" s="3" t="s">
+      <c r="AE7" s="16" t="s">
         <v>86</v>
       </c>
       <c r="AF7" s="10"/>
@@ -1345,7 +1344,7 @@
       <c r="AD8" s="3">
         <v>350</v>
       </c>
-      <c r="AE8" s="3" t="s">
+      <c r="AE8" s="16" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1384,7 +1383,7 @@
       <c r="Y9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AA9" s="17">
+      <c r="AA9" s="16">
         <f>SUM(Z7:Z8)</f>
         <v>2300</v>
       </c>
@@ -1395,7 +1394,7 @@
       <c r="AD9" s="3">
         <v>80</v>
       </c>
-      <c r="AE9" s="3" t="s">
+      <c r="AE9" s="16" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1470,7 +1469,7 @@
       <c r="Y11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AA11" s="17">
+      <c r="AA11" s="16">
         <v>3000</v>
       </c>
       <c r="AB11" s="4"/>
@@ -1480,7 +1479,7 @@
       <c r="AD11" s="3">
         <v>120</v>
       </c>
-      <c r="AE11" s="3" t="s">
+      <c r="AE11" s="16" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1514,7 +1513,7 @@
         <v>77</v>
       </c>
       <c r="AE12" s="3" t="s">
-        <v>88</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.3">
@@ -1542,7 +1541,7 @@
       <c r="Y13" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AA13" s="17">
+      <c r="AA13" s="16">
         <v>1000</v>
       </c>
       <c r="AB13" s="4"/>
@@ -1553,7 +1552,7 @@
         <v>150</v>
       </c>
       <c r="AE13" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.3">
@@ -1580,13 +1579,13 @@
       <c r="X14" s="4"/>
       <c r="AB14" s="4"/>
       <c r="AC14" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD14" s="3">
         <v>154</v>
       </c>
-      <c r="AE14" s="3" t="s">
-        <v>113</v>
+      <c r="AE14" s="16" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.3">
@@ -1620,12 +1619,12 @@
       </c>
       <c r="AB15" s="4"/>
       <c r="AC15" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AD15" s="3">
         <v>301</v>
       </c>
-      <c r="AE15" s="3" t="s">
+      <c r="AE15" s="16" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1694,7 +1693,7 @@
       <c r="U18" s="4"/>
       <c r="X18" s="4"/>
       <c r="Y18" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Z18" s="3">
         <v>-150</v>
@@ -1718,7 +1717,7 @@
       <c r="U19" s="4"/>
       <c r="X19" s="4"/>
       <c r="Y19" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Z19" s="3">
         <v>77</v>
@@ -1771,7 +1770,7 @@
       <c r="Y21" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="AA21" s="17">
+      <c r="AA21" s="16">
         <f>SUM(Z15:Z20)</f>
         <v>3272</v>
       </c>
@@ -1799,9 +1798,9 @@
       <c r="C23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="K23" s="19">
+        <v>128</v>
+      </c>
+      <c r="K23" s="18">
         <f>(الأرصدة!AA2)-1667</f>
         <v>1258</v>
       </c>
@@ -1818,7 +1817,7 @@
       <c r="Y23" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="AA23" s="3">
+      <c r="AA23" s="16">
         <f>L27</f>
         <v>820</v>
       </c>
@@ -1839,9 +1838,9 @@
       <c r="U25" s="4"/>
       <c r="X25" s="4"/>
       <c r="Y25" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA25" s="17">
+        <v>89</v>
+      </c>
+      <c r="AA25" s="16">
         <v>2000</v>
       </c>
       <c r="AB25" s="4"/>
@@ -1880,9 +1879,9 @@
       <c r="U27" s="3"/>
       <c r="X27" s="3"/>
       <c r="Y27" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA27" s="16">
+        <v>90</v>
+      </c>
+      <c r="AA27" s="15">
         <f>T2</f>
         <v>0</v>
       </c>
@@ -1903,9 +1902,9 @@
       <c r="U29" s="3"/>
       <c r="X29" s="3"/>
       <c r="Y29" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="AA29" s="18">
+        <v>91</v>
+      </c>
+      <c r="AA29" s="17">
         <f>M27</f>
         <v>2752</v>
       </c>
@@ -1922,10 +1921,10 @@
     <row r="31" spans="3:28" ht="46" x14ac:dyDescent="0.3">
       <c r="C31" s="3"/>
       <c r="D31" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3" t="s">
@@ -1944,9 +1943,9 @@
       <c r="U31" s="3"/>
       <c r="X31" s="3"/>
       <c r="Y31" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA31" s="17">
+        <v>93</v>
+      </c>
+      <c r="AA31" s="16">
         <f>W2</f>
         <v>22024</v>
       </c>
@@ -1985,12 +1984,12 @@
     </row>
     <row r="33" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y33" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="34" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y34" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Z34" s="3">
         <v>0</v>
@@ -2004,9 +2003,9 @@
     </row>
     <row r="36" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y36" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="AA36" s="3">
+        <v>144</v>
+      </c>
+      <c r="AA36" s="16">
         <v>1667</v>
       </c>
     </row>
@@ -2033,7 +2032,7 @@
     </row>
     <row r="40" spans="3:28" ht="46" x14ac:dyDescent="0.3">
       <c r="Y40" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="AA40" s="3">
         <f>SUM(Z38:Z39)</f>
@@ -2079,7 +2078,7 @@
       <c r="U44" s="3"/>
       <c r="X44" s="3"/>
       <c r="Y44" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Z44" s="3">
         <v>-200</v>
@@ -2093,7 +2092,7 @@
       <c r="U45" s="3"/>
       <c r="X45" s="3"/>
       <c r="Y45" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Z45" s="3">
         <f>AA40</f>
@@ -2103,7 +2102,7 @@
     </row>
     <row r="46" spans="3:28" x14ac:dyDescent="0.3">
       <c r="Y46" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AA46" s="3">
         <f>SUM(Z42:Z45)</f>
@@ -2208,27 +2207,27 @@
       <c r="U1" s="3"/>
       <c r="V1" s="2"/>
       <c r="W1" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="Z1" s="4"/>
       <c r="AA1" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="AB1" s="3"/>
       <c r="AD1" s="3" t="s">
         <v>49</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="AF1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="AH1" s="4"/>
     </row>
@@ -2275,12 +2274,12 @@
         <v>9963</v>
       </c>
       <c r="X2" s="11">
-        <f>(1500+(303*3))+5001</f>
-        <v>7410</v>
+        <f>AE27</f>
+        <v>7409</v>
       </c>
       <c r="Y2" s="11">
         <f>SUM(W2:X2)</f>
-        <v>17373</v>
+        <v>17372</v>
       </c>
       <c r="Z2" s="4"/>
       <c r="AA2" s="11">
@@ -2295,11 +2294,11 @@
       </c>
       <c r="AE2" s="3">
         <f>SUM(AE6:AE20)</f>
-        <v>1712</v>
+        <v>4637</v>
       </c>
       <c r="AF2" s="3">
         <f>SUM(AF6:AF20)</f>
-        <v>8018</v>
+        <v>5093</v>
       </c>
       <c r="AG2" s="3">
         <f>SUM(AG6:AG20)</f>
@@ -2417,13 +2416,13 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="4"/>
       <c r="AA5" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="AB5" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="AC5" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
@@ -2471,7 +2470,7 @@
         <v>39948</v>
       </c>
       <c r="R6" s="4"/>
-      <c r="S6">
+      <c r="S6" s="3">
         <v>1</v>
       </c>
       <c r="T6" s="3" t="s">
@@ -2485,7 +2484,7 @@
         <v>4</v>
       </c>
       <c r="X6" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Y6" s="11">
         <v>200</v>
@@ -2495,22 +2494,22 @@
         <v>3</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="AC6" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AD6" s="3">
         <v>902</v>
       </c>
       <c r="AE6" s="3">
-        <v>601</v>
+        <v>902</v>
       </c>
       <c r="AF6" s="3">
         <f>AD6-AE6</f>
-        <v>301</v>
-      </c>
-      <c r="AG6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="3">
         <v>301</v>
       </c>
       <c r="AH6" s="4"/>
@@ -2553,7 +2552,7 @@
         <v>864</v>
       </c>
       <c r="R7" s="4"/>
-      <c r="S7">
+      <c r="S7" s="3">
         <v>1</v>
       </c>
       <c r="T7" s="3" t="s">
@@ -2567,7 +2566,7 @@
         <v>4</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Y7" s="11">
         <v>500</v>
@@ -2577,20 +2576,20 @@
         <v>4</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AC7" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AD7" s="3">
         <v>1995</v>
       </c>
       <c r="AE7" s="3">
-        <v>499</v>
+        <v>998</v>
       </c>
       <c r="AF7" s="3">
         <f>AD7-AE7</f>
-        <v>1496</v>
+        <v>997</v>
       </c>
       <c r="AG7" s="3">
         <v>499</v>
@@ -2631,13 +2630,13 @@
         <v>1</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Q8" s="11">
         <v>17777</v>
       </c>
       <c r="R8" s="4"/>
-      <c r="S8">
+      <c r="S8" s="3">
         <v>1</v>
       </c>
       <c r="T8" s="3" t="s">
@@ -2651,7 +2650,7 @@
         <v>4</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Y8" s="11">
         <v>303</v>
@@ -2661,22 +2660,22 @@
         <v>4</v>
       </c>
       <c r="AB8" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC8" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AD8" s="3">
         <v>616</v>
       </c>
       <c r="AE8" s="3">
-        <v>308</v>
+        <v>462</v>
       </c>
       <c r="AF8" s="3">
         <f>AD8-AE8</f>
-        <v>308</v>
-      </c>
-      <c r="AG8" s="11">
+        <v>154</v>
+      </c>
+      <c r="AG8" s="3">
         <v>154</v>
       </c>
       <c r="AH8" s="4"/>
@@ -2721,7 +2720,7 @@
         <v>1676</v>
       </c>
       <c r="R9" s="4"/>
-      <c r="S9">
+      <c r="S9" s="3">
         <v>1</v>
       </c>
       <c r="T9" s="3" t="s">
@@ -2735,7 +2734,7 @@
         <v>4</v>
       </c>
       <c r="X9" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Y9" s="11">
         <v>750</v>
@@ -2745,22 +2744,22 @@
         <v>4</v>
       </c>
       <c r="AB9" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AC9" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AD9" s="3">
         <v>1216</v>
       </c>
       <c r="AE9" s="3">
-        <v>304</v>
+        <v>608</v>
       </c>
       <c r="AF9" s="3">
         <f>AD9-AE9</f>
-        <v>912</v>
-      </c>
-      <c r="AG9" s="11">
+        <v>608</v>
+      </c>
+      <c r="AG9" s="3">
         <v>304</v>
       </c>
       <c r="AH9" s="4"/>
@@ -2799,7 +2798,7 @@
         <v>787</v>
       </c>
       <c r="R10" s="4"/>
-      <c r="S10">
+      <c r="S10" s="3">
         <v>1</v>
       </c>
       <c r="T10" s="3" t="s">
@@ -2813,7 +2812,7 @@
         <v>4</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Y10" s="11">
         <v>188</v>
@@ -2823,23 +2822,23 @@
         <v>4</v>
       </c>
       <c r="AB10" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="AC10" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="AD10" s="15">
+        <v>102</v>
+      </c>
+      <c r="AD10" s="3">
         <f>AG10*3</f>
         <v>5001</v>
       </c>
       <c r="AE10" s="3">
-        <v>0</v>
+        <v>1667</v>
       </c>
       <c r="AF10" s="3">
         <f>AD10-AE10</f>
-        <v>5001</v>
-      </c>
-      <c r="AG10" s="11">
+        <v>3334</v>
+      </c>
+      <c r="AG10" s="3">
         <f>1618+49</f>
         <v>1667</v>
       </c>
@@ -2871,13 +2870,13 @@
         <v>4</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q11" s="11">
         <v>2000</v>
       </c>
       <c r="R11" s="4"/>
-      <c r="S11">
+      <c r="S11" s="3">
         <v>1</v>
       </c>
       <c r="T11" s="3" t="s">
@@ -2891,7 +2890,7 @@
         <v>4</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Y11" s="11">
         <v>200</v>
@@ -2936,11 +2935,11 @@
         <v>7027</v>
       </c>
       <c r="R12" s="4"/>
-      <c r="S12">
+      <c r="S12" s="3">
         <v>2</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U12" s="11">
         <v>10000</v>
@@ -2950,7 +2949,7 @@
         <v>4</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Y12" s="11">
         <v>200</v>
@@ -2989,11 +2988,11 @@
       <c r="P13" s="3"/>
       <c r="Q13" s="11"/>
       <c r="R13" s="4"/>
-      <c r="S13">
+      <c r="S13" s="3">
         <v>2</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="U13" s="11">
         <v>1000</v>
@@ -3003,7 +3002,7 @@
         <v>4</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="Y13" s="11">
         <v>223</v>
@@ -3040,11 +3039,11 @@
       <c r="P14" s="3"/>
       <c r="Q14" s="11"/>
       <c r="R14" s="4"/>
-      <c r="S14">
+      <c r="S14" s="3">
         <v>2</v>
       </c>
       <c r="T14" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U14" s="11">
         <v>500</v>
@@ -3054,7 +3053,7 @@
         <v>4</v>
       </c>
       <c r="X14" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Y14" s="11">
         <v>501</v>
@@ -3095,7 +3094,7 @@
         <v>3</v>
       </c>
       <c r="T15" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="U15" s="3">
         <v>3701</v>
@@ -3105,7 +3104,7 @@
         <v>4</v>
       </c>
       <c r="X15" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Y15" s="11">
         <v>1500</v>
@@ -3146,7 +3145,7 @@
         <v>3</v>
       </c>
       <c r="T16" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="U16" s="3">
         <v>1000</v>
@@ -3156,7 +3155,7 @@
         <v>4</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Y16" s="11"/>
       <c r="Z16" s="4"/>
@@ -3195,7 +3194,7 @@
         <v>3</v>
       </c>
       <c r="T17" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="U17" s="11">
         <v>850</v>
@@ -3205,7 +3204,7 @@
         <v>10</v>
       </c>
       <c r="X17" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="Y17" s="11">
         <v>2734</v>
@@ -3245,7 +3244,7 @@
       <c r="S18" s="3">
         <v>4</v>
       </c>
-      <c r="T18" s="15" t="str">
+      <c r="T18" s="3" t="str">
         <f>W1</f>
         <v>سفرة مصر</v>
       </c>
@@ -3258,7 +3257,7 @@
         <v>4</v>
       </c>
       <c r="X18" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="Y18" s="3">
         <v>228</v>
@@ -3301,7 +3300,7 @@
         <v>4</v>
       </c>
       <c r="X19" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="Y19" s="5">
         <v>1957</v>
@@ -3342,7 +3341,7 @@
         <v>4</v>
       </c>
       <c r="X20" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="Y20" s="11">
         <v>479</v>
@@ -3464,6 +3463,19 @@
       <c r="W24" s="4"/>
       <c r="X24" s="4"/>
       <c r="Y24" s="4"/>
+      <c r="AB24" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="AC24">
+        <v>1995</v>
+      </c>
+      <c r="AD24">
+        <v>499</v>
+      </c>
+      <c r="AE24">
+        <f>AC24-AD24</f>
+        <v>1496</v>
+      </c>
     </row>
     <row r="25" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C25" s="3"/>
@@ -3490,6 +3502,19 @@
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
+      <c r="AB25" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="AC25">
+        <v>1216</v>
+      </c>
+      <c r="AD25" s="3">
+        <v>304</v>
+      </c>
+      <c r="AE25">
+        <f>AC25-AD25</f>
+        <v>912</v>
+      </c>
     </row>
     <row r="26" spans="2:34" ht="22" x14ac:dyDescent="0.3">
       <c r="C26" s="3"/>
@@ -3517,7 +3542,17 @@
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
       <c r="Y26" t="s">
-        <v>99</v>
+        <v>98</v>
+      </c>
+      <c r="AB26" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="AC26">
+        <v>5001</v>
+      </c>
+      <c r="AE26">
+        <f>AC26-AD26</f>
+        <v>5001</v>
       </c>
     </row>
     <row r="27" spans="2:34" ht="22" x14ac:dyDescent="0.3">
@@ -3531,7 +3566,7 @@
       <c r="J27" s="3"/>
       <c r="K27" s="4"/>
       <c r="L27" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M27" s="6">
         <v>-10500</v>
@@ -3550,6 +3585,10 @@
       <c r="Y27" s="12">
         <f>M29-W27</f>
         <v>-1915</v>
+      </c>
+      <c r="AE27">
+        <f>SUM(AE24:AE26)</f>
+        <v>7409</v>
       </c>
     </row>
     <row r="28" spans="2:34" ht="22" x14ac:dyDescent="0.3">

</xml_diff>